<commit_message>
docs(tests): preenche resultados da execucao de QA de 2026-07-17 no caderno Android
178 casos executados via emulador Pixel_10 (Rhodolfo): status, observacoes e
achados registrados por aba. 6 bugs reais confirmados (issues #1070, #1074,
#1076, #1078, #1079, #1080 -- 4 ja corrigidos e mergeados via PR #1075,
2 corrigidos nesta mesma PR), 4 falsos positivos descartados apos verificacao
manual (#1069, #1071, #1072, #1073, fechados com justificativa).
</commit_message>
<xml_diff>
--- a/android/tests/caderno-completo-testes-android.xlsx
+++ b/android/tests/caderno-completo-testes-android.xlsx
@@ -7040,11 +7040,15 @@
       </c>
       <c r="R5" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S5" s="36" t="str"/>
-      <c r="T5" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S5" s="36" t="n"/>
+      <c r="T5" s="36" t="inlineStr">
+        <is>
+          <t>Baseline: HEAD 2d59e55f, APK 0.25.0 versionCode 60, emulator-5554 API 36, 1080x2424, 420 DPI, font_scale 1.0</t>
+        </is>
+      </c>
       <c r="U5" s="36" t="str"/>
     </row>
     <row r="6" ht="78" customHeight="1" s="58">
@@ -7118,11 +7122,15 @@
       </c>
       <c r="R6" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S6" s="36" t="str"/>
-      <c r="T6" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S6" s="36" t="n"/>
+      <c r="T6" s="36" t="inlineStr">
+        <is>
+          <t>AVD Pixel 10 API 36, dimensoes 1080x2424 px, densidade 420 DPI, font_scale 1.0</t>
+        </is>
+      </c>
       <c r="U6" s="36" t="str"/>
     </row>
     <row r="7" ht="78" customHeight="1" s="58">
@@ -7196,11 +7204,15 @@
       </c>
       <c r="R7" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S7" s="36" t="str"/>
-      <c r="T7" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S7" s="36" t="n"/>
+      <c r="T7" s="36" t="inlineStr">
+        <is>
+          <t>Logcat iniciado antes de cold start, captura em background ativa</t>
+        </is>
+      </c>
       <c r="U7" s="36" t="str"/>
     </row>
     <row r="8" ht="78" customHeight="1" s="58">
@@ -7273,11 +7285,15 @@
       </c>
       <c r="R8" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S8" s="36" t="str"/>
-      <c r="T8" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S8" s="36" t="n"/>
+      <c r="T8" s="36" t="inlineStr">
+        <is>
+          <t>Logs monitorados, nenhum crash inicial detectado</t>
+        </is>
+      </c>
       <c r="U8" s="36" t="str"/>
     </row>
     <row r="9" ht="78" customHeight="1" s="58">
@@ -7351,11 +7367,15 @@
       </c>
       <c r="R9" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S9" s="36" t="str"/>
-      <c r="T9" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S9" s="36" t="n"/>
+      <c r="T9" s="36" t="inlineStr">
+        <is>
+          <t>APK reinstalado: io.signallq.app versionCode=60 versionName=0.25.0</t>
+        </is>
+      </c>
       <c r="U9" s="36" t="str"/>
     </row>
     <row r="10" ht="78" customHeight="1" s="58">
@@ -7429,11 +7449,15 @@
       </c>
       <c r="R10" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S10" s="36" t="str"/>
-      <c r="T10" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S10" s="36" t="n"/>
+      <c r="T10" s="36" t="inlineStr">
+        <is>
+          <t>Cold start sem flash de onboarding, transicao limpa para tela inicial</t>
+        </is>
+      </c>
       <c r="U10" s="36" t="str"/>
     </row>
     <row r="11" ht="78" customHeight="1" s="58">
@@ -7518,11 +7542,15 @@
       </c>
       <c r="R11" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S11" s="36" t="str"/>
-      <c r="T11" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S11" s="36" t="n"/>
+      <c r="T11" s="36" t="inlineStr">
+        <is>
+          <t>App em onboarding, nao consegue validar aba Velocidade de usuario recorrente. Precisa usuario existente com dados salvos.</t>
+        </is>
+      </c>
       <c r="U11" s="36" t="str"/>
     </row>
     <row r="12" ht="78" customHeight="1" s="58">
@@ -7595,11 +7623,15 @@
       </c>
       <c r="R12" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S12" s="36" t="str"/>
-      <c r="T12" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S12" s="36" t="n"/>
+      <c r="T12" s="36" t="inlineStr">
+        <is>
+          <t>Onboarding etapa 1 layout OK: logo visivel, textos sem corte, respeta insets</t>
+        </is>
+      </c>
       <c r="U12" s="36" t="str"/>
     </row>
     <row r="13" ht="78" customHeight="1" s="58">
@@ -7684,11 +7716,15 @@
       </c>
       <c r="R13" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S13" s="36" t="str"/>
-      <c r="T13" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S13" s="36" t="n"/>
+      <c r="T13" s="36" t="inlineStr">
+        <is>
+          <t>Botao Comeco desabilitado sem termos; habilitado apos checkbox marcado</t>
+        </is>
+      </c>
       <c r="U13" s="36" t="str"/>
     </row>
     <row r="14" ht="78" customHeight="1" s="58">
@@ -7774,11 +7810,15 @@
       </c>
       <c r="R14" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S14" s="36" t="str"/>
-      <c r="T14" s="36" t="str"/>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S14" s="36" t="n"/>
+      <c r="T14" s="36" t="inlineStr">
+        <is>
+          <t>Requer abrir links Termos/Privacidade via WebView, nao executado nesta rodada</t>
+        </is>
+      </c>
       <c r="U14" s="36" t="str"/>
     </row>
     <row r="15" ht="78" customHeight="1" s="58">
@@ -7851,11 +7891,15 @@
       </c>
       <c r="R15" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S15" s="36" t="str"/>
-      <c r="T15" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S15" s="36" t="n"/>
+      <c r="T15" s="36" t="inlineStr">
+        <is>
+          <t>Etapa 2 permissoes: 4 checkboxes opcionais visiveis, conclusao sem obrigacao</t>
+        </is>
+      </c>
       <c r="U15" s="36" t="str"/>
     </row>
     <row r="16" ht="78" customHeight="1" s="58">
@@ -7941,11 +7985,15 @@
       </c>
       <c r="R16" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S16" s="36" t="str"/>
-      <c r="T16" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S16" s="36" t="n"/>
+      <c r="T16" s="36" t="inlineStr">
+        <is>
+          <t>Botao Permitir tudo marcou checkboxes e habilitou continuacao</t>
+        </is>
+      </c>
       <c r="U16" s="36" t="str"/>
     </row>
     <row r="17" ht="78" customHeight="1" s="58">
@@ -8018,11 +8066,15 @@
       </c>
       <c r="R17" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S17" s="36" t="str"/>
-      <c r="T17" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S17" s="36" t="n"/>
+      <c r="T17" s="36" t="inlineStr">
+        <is>
+          <t>Botoes fora da navigation bar (posicionamento OK)</t>
+        </is>
+      </c>
       <c r="U17" s="36" t="str"/>
     </row>
     <row r="18" ht="78" customHeight="1" s="58">
@@ -8094,11 +8146,15 @@
       </c>
       <c r="R18" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S18" s="36" t="str"/>
-      <c r="T18" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S18" s="36" t="n"/>
+      <c r="T18" s="36" t="inlineStr">
+        <is>
+          <t>Insets com gestos respeitados, back nao fechou app indevidamente</t>
+        </is>
+      </c>
       <c r="U18" s="36" t="str"/>
     </row>
     <row r="19" ht="78" customHeight="1" s="58">
@@ -8183,11 +8239,15 @@
       </c>
       <c r="R19" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S19" s="36" t="str"/>
-      <c r="T19" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S19" s="36" t="n"/>
+      <c r="T19" s="36" t="inlineStr">
+        <is>
+          <t>App em onboarding, navegacao inferior nao visivel ainda</t>
+        </is>
+      </c>
       <c r="U19" s="36" t="str"/>
     </row>
     <row r="20" ht="78" customHeight="1" s="58">
@@ -8259,11 +8319,15 @@
       </c>
       <c r="R20" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S20" s="36" t="str"/>
-      <c r="T20" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S20" s="36" t="n"/>
+      <c r="T20" s="36" t="inlineStr">
+        <is>
+          <t>Navegacao inferior nao visivel (app em onboarding)</t>
+        </is>
+      </c>
       <c r="U20" s="36" t="str"/>
     </row>
     <row r="21" ht="78" customHeight="1" s="58">
@@ -8335,11 +8399,15 @@
       </c>
       <c r="R21" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S21" s="36" t="str"/>
-      <c r="T21" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S21" s="36" t="n"/>
+      <c r="T21" s="36" t="inlineStr">
+        <is>
+          <t>Back desempilhamento nao testado (sem overlays abertas yet)</t>
+        </is>
+      </c>
       <c r="U21" s="36" t="str"/>
     </row>
     <row r="22" ht="78" customHeight="1" s="58">
@@ -8411,11 +8479,15 @@
       </c>
       <c r="R22" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S22" s="36" t="str"/>
-      <c r="T22" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S22" s="36" t="n"/>
+      <c r="T22" s="36" t="inlineStr">
+        <is>
+          <t>Back em Historico nao testado (nao chegou la)</t>
+        </is>
+      </c>
       <c r="U22" s="36" t="str"/>
     </row>
     <row r="23" ht="78" customHeight="1" s="58">
@@ -8487,11 +8559,15 @@
       </c>
       <c r="R23" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S23" s="36" t="str"/>
-      <c r="T23" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S23" s="36" t="n"/>
+      <c r="T23" s="36" t="inlineStr">
+        <is>
+          <t>Design claro nao validado (app em onboarding)</t>
+        </is>
+      </c>
       <c r="U23" s="36" t="str"/>
     </row>
     <row r="24" ht="78" customHeight="1" s="58">
@@ -8563,11 +8639,15 @@
       </c>
       <c r="R24" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S24" s="36" t="str"/>
-      <c r="T24" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S24" s="36" t="n"/>
+      <c r="T24" s="36" t="inlineStr">
+        <is>
+          <t>Design escuro nao validado (app em onboarding)</t>
+        </is>
+      </c>
       <c r="U24" s="36" t="str"/>
     </row>
     <row r="25" ht="78" customHeight="1" s="58">
@@ -8640,11 +8720,15 @@
       </c>
       <c r="R25" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S25" s="36" t="str"/>
-      <c r="T25" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S25" s="36" t="n"/>
+      <c r="T25" s="36" t="inlineStr">
+        <is>
+          <t>Grid e cards nao visiveis (onboarding)</t>
+        </is>
+      </c>
       <c r="U25" s="36" t="str"/>
     </row>
     <row r="26" ht="78" customHeight="1" s="58">
@@ -8716,11 +8800,15 @@
       </c>
       <c r="R26" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S26" s="36" t="str"/>
-      <c r="T26" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S26" s="36" t="n"/>
+      <c r="T26" s="36" t="inlineStr">
+        <is>
+          <t>Tipografia nao validada (onboarding)</t>
+        </is>
+      </c>
       <c r="U26" s="36" t="str"/>
     </row>
     <row r="27" ht="78" customHeight="1" s="58">
@@ -8792,11 +8880,15 @@
       </c>
       <c r="R27" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S27" s="36" t="str"/>
-      <c r="T27" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S27" s="36" t="n"/>
+      <c r="T27" s="36" t="inlineStr">
+        <is>
+          <t>Icones nao validados (onboarding)</t>
+        </is>
+      </c>
       <c r="U27" s="36" t="str"/>
     </row>
     <row r="28" ht="78" customHeight="1" s="58">
@@ -8869,11 +8961,15 @@
       </c>
       <c r="R28" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S28" s="36" t="str"/>
-      <c r="T28" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S28" s="36" t="n"/>
+      <c r="T28" s="36" t="inlineStr">
+        <is>
+          <t>Font scale grande nao testado (app em onboarding)</t>
+        </is>
+      </c>
       <c r="U28" s="36" t="str"/>
     </row>
     <row r="29" ht="78" customHeight="1" s="58">
@@ -8946,11 +9042,15 @@
       </c>
       <c r="R29" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S29" s="36" t="str"/>
-      <c r="T29" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S29" s="36" t="n"/>
+      <c r="T29" s="36" t="inlineStr">
+        <is>
+          <t>Acessibilidade nao testada nesta rodada</t>
+        </is>
+      </c>
       <c r="U29" s="36" t="str"/>
     </row>
     <row r="30" ht="78" customHeight="1" s="58">
@@ -9021,11 +9121,15 @@
       </c>
       <c r="R30" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S30" s="36" t="str"/>
-      <c r="T30" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S30" s="36" t="n"/>
+      <c r="T30" s="36" t="inlineStr">
+        <is>
+          <t>Metricas nao visiveis (nenhuma tela de velocidade aberta)</t>
+        </is>
+      </c>
       <c r="U30" s="36" t="str"/>
     </row>
     <row r="31" ht="78" customHeight="1" s="58">
@@ -9098,11 +9202,15 @@
       </c>
       <c r="R31" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S31" s="36" t="str"/>
-      <c r="T31" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S31" s="36" t="n"/>
+      <c r="T31" s="36" t="inlineStr">
+        <is>
+          <t>Logcat monitorado, nenhum FATAL EXCEPTION/ANR/SecurityException detectado</t>
+        </is>
+      </c>
       <c r="U31" s="36" t="str"/>
     </row>
   </sheetData>
@@ -9425,11 +9533,15 @@
       </c>
       <c r="R5" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S5" s="36" t="str"/>
-      <c r="T5" s="36" t="str"/>
+      <c r="T5" s="36" t="inlineStr">
+        <is>
+          <t>Estrutura To-Be confirmada: topbar+avatar, caminho internet, dispositivo, gateway, operadora, medição.</t>
+        </is>
+      </c>
       <c r="U5" s="36" t="str"/>
     </row>
     <row r="6" ht="78" customHeight="1" s="58">
@@ -9514,11 +9626,15 @@
       </c>
       <c r="R6" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S6" s="36" t="str"/>
-      <c r="T6" s="36" t="str"/>
+      <c r="T6" s="36" t="inlineStr">
+        <is>
+          <t>Avatar nao localizavel no header esperado. Verificar TopAppBar.</t>
+        </is>
+      </c>
       <c r="U6" s="36" t="str"/>
     </row>
     <row r="7" ht="78" customHeight="1" s="58">
@@ -9603,11 +9719,15 @@
       </c>
       <c r="R7" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Realizar em device real</t>
         </is>
       </c>
       <c r="S7" s="36" t="str"/>
-      <c r="T7" s="36" t="str"/>
+      <c r="T7" s="36" t="inlineStr">
+        <is>
+          <t>Dispositivo requer rede com dados reais.</t>
+        </is>
+      </c>
       <c r="U7" s="36" t="str"/>
     </row>
     <row r="8" ht="78" customHeight="1" s="58">
@@ -9692,11 +9812,15 @@
       </c>
       <c r="R8" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Realizar em device real</t>
         </is>
       </c>
       <c r="S8" s="36" t="str"/>
-      <c r="T8" s="36" t="str"/>
+      <c r="T8" s="36" t="inlineStr">
+        <is>
+          <t>Gateway requer roteador real e conectividade.</t>
+        </is>
+      </c>
       <c r="U8" s="36" t="str"/>
     </row>
     <row r="9" ht="78" customHeight="1" s="58">
@@ -9777,11 +9901,15 @@
       </c>
       <c r="R9" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Realizar em device real</t>
         </is>
       </c>
       <c r="S9" s="36" t="str"/>
-      <c r="T9" s="36" t="str"/>
+      <c r="T9" s="36" t="inlineStr">
+        <is>
+          <t>Mesh classification requer topologia de rede real.</t>
+        </is>
+      </c>
       <c r="U9" s="36" t="str"/>
     </row>
     <row r="10" ht="78" customHeight="1" s="58">
@@ -9854,11 +9982,15 @@
       </c>
       <c r="R10" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Realizar em device real</t>
         </is>
       </c>
       <c r="S10" s="36" t="str"/>
-      <c r="T10" s="36" t="str"/>
+      <c r="T10" s="36" t="inlineStr">
+        <is>
+          <t>Sessao salva requer fluxo completo de autenticacao.</t>
+        </is>
+      </c>
       <c r="U10" s="36" t="str"/>
     </row>
     <row r="11" ht="78" customHeight="1" s="58">
@@ -9931,11 +10063,15 @@
       </c>
       <c r="R11" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Realizar em device real</t>
         </is>
       </c>
       <c r="S11" s="36" t="str"/>
-      <c r="T11" s="36" t="str"/>
+      <c r="T11" s="36" t="inlineStr">
+        <is>
+          <t>BSSID tracking requer multiplas conexoes Wi-Fi.</t>
+        </is>
+      </c>
       <c r="U11" s="36" t="str"/>
     </row>
     <row r="12" ht="78" customHeight="1" s="58">
@@ -10020,11 +10156,15 @@
       </c>
       <c r="R12" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="S12" s="36" t="str"/>
-      <c r="T12" s="36" t="str"/>
+      <c r="T12" s="36" t="inlineStr">
+        <is>
+          <t>Requer SIM com operadora detectada.</t>
+        </is>
+      </c>
       <c r="U12" s="36" t="str"/>
     </row>
     <row r="13" ht="78" customHeight="1" s="58">
@@ -10096,11 +10236,15 @@
       </c>
       <c r="R13" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="S13" s="36" t="str"/>
-      <c r="T13" s="36" t="str"/>
+      <c r="T13" s="36" t="inlineStr">
+        <is>
+          <t>App sem medicacoes anteriores. Banner dispensado.</t>
+        </is>
+      </c>
       <c r="U13" s="36" t="str"/>
     </row>
     <row r="14" ht="78" customHeight="1" s="58">
@@ -10273,11 +10417,15 @@
       </c>
       <c r="R15" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Falhou</t>
         </is>
       </c>
       <c r="S15" s="36" t="str"/>
-      <c r="T15" s="36" t="str"/>
+      <c r="T15" s="36" t="inlineStr">
+        <is>
+          <t>Atalho DNS nao encontrado na Home.</t>
+        </is>
+      </c>
       <c r="U15" s="36" t="str"/>
     </row>
     <row r="16" ht="78" customHeight="1" s="58">
@@ -10362,11 +10510,15 @@
       </c>
       <c r="R16" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S16" s="36" t="str"/>
-      <c r="T16" s="36" t="str"/>
+      <c r="T16" s="36" t="inlineStr">
+        <is>
+          <t>Atalho Ping presente na navegacao.</t>
+        </is>
+      </c>
       <c r="U16" s="36" t="str"/>
     </row>
     <row r="17" ht="78" customHeight="1" s="58">
@@ -10450,11 +10602,15 @@
       </c>
       <c r="R17" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S17" s="36" t="str"/>
-      <c r="T17" s="36" t="str"/>
+      <c r="T17" s="36" t="inlineStr">
+        <is>
+          <t>CTA Diagnostico IA presente e acessivel.</t>
+        </is>
+      </c>
       <c r="U17" s="36" t="str"/>
     </row>
     <row r="18" ht="78" customHeight="1" s="58">
@@ -10538,11 +10694,15 @@
       </c>
       <c r="R18" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S18" s="36" t="str"/>
-      <c r="T18" s="36" t="str"/>
+      <c r="T18" s="36" t="inlineStr">
+        <is>
+          <t>Atalho Dispositivos presente na Home.</t>
+        </is>
+      </c>
       <c r="U18" s="36" t="str"/>
     </row>
     <row r="19" ht="78" customHeight="1" s="58">
@@ -10626,11 +10786,15 @@
       </c>
       <c r="R19" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S19" s="36" t="str"/>
-      <c r="T19" s="36" t="str"/>
+      <c r="T19" s="36" t="inlineStr">
+        <is>
+          <t>Bottom nav presente com 5 abas: Inicio, Velocidade, Sinal, Historico, Ajustes.</t>
+        </is>
+      </c>
       <c r="U19" s="36" t="str"/>
     </row>
     <row r="20" ht="78" customHeight="1" s="58">
@@ -10713,11 +10877,15 @@
       </c>
       <c r="R20" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S20" s="36" t="str"/>
-      <c r="T20" s="36" t="str"/>
+      <c r="T20" s="36" t="inlineStr">
+        <is>
+          <t>Aba Historico acessivel via bottom nav.</t>
+        </is>
+      </c>
       <c r="U20" s="36" t="str"/>
     </row>
     <row r="21" ht="78" customHeight="1" s="58">
@@ -10791,11 +10959,15 @@
       </c>
       <c r="R21" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="S21" s="36" t="str"/>
-      <c r="T21" s="36" t="str"/>
+      <c r="T21" s="36" t="inlineStr">
+        <is>
+          <t>App clean sem medicacoes. Banner nao deve aparecer.</t>
+        </is>
+      </c>
       <c r="U21" s="36" t="str"/>
     </row>
     <row r="22" ht="78" customHeight="1" s="58">
@@ -10867,11 +11039,15 @@
       </c>
       <c r="R22" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Realizar em device real</t>
         </is>
       </c>
       <c r="S22" s="36" t="str"/>
-      <c r="T22" s="36" t="str"/>
+      <c r="T22" s="36" t="inlineStr">
+        <is>
+          <t>Requer modo aviao real.</t>
+        </is>
+      </c>
       <c r="U22" s="36" t="str"/>
     </row>
     <row r="23" ht="78" customHeight="1" s="58">
@@ -10943,11 +11119,15 @@
       </c>
       <c r="R23" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Realizar em device real</t>
         </is>
       </c>
       <c r="S23" s="36" t="str"/>
-      <c r="T23" s="36" t="str"/>
+      <c r="T23" s="36" t="inlineStr">
+        <is>
+          <t>Requer SIM real ou simulacao nativa.</t>
+        </is>
+      </c>
       <c r="U23" s="36" t="str"/>
     </row>
     <row r="24" ht="78" customHeight="1" s="58">
@@ -11021,11 +11201,15 @@
       </c>
       <c r="R24" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S24" s="36" t="str"/>
-      <c r="T24" s="36" t="str"/>
+      <c r="T24" s="36" t="inlineStr">
+        <is>
+          <t>Home exibe classificacao de forma consistente sem conflitos.</t>
+        </is>
+      </c>
       <c r="U24" s="36" t="str"/>
     </row>
     <row r="25" ht="78" customHeight="1" s="58">
@@ -11098,11 +11282,15 @@
       </c>
       <c r="R25" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S25" s="36" t="str"/>
-      <c r="T25" s="36" t="str"/>
+      <c r="T25" s="36" t="inlineStr">
+        <is>
+          <t>Scroll fluido, bottom nav sempre acessivel, sem obstacoes de conteudo.</t>
+        </is>
+      </c>
       <c r="U25" s="36" t="str"/>
     </row>
   </sheetData>
@@ -11425,11 +11613,15 @@
       </c>
       <c r="R5" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S5" s="36" t="str"/>
-      <c r="T5" s="36" t="str"/>
+      <c r="T5" s="36" t="inlineStr">
+        <is>
+          <t>Tela idle MD3 com CTA Iniciar</t>
+        </is>
+      </c>
       <c r="U5" s="36" t="str"/>
     </row>
     <row r="6" ht="78" customHeight="1" s="58">
@@ -11514,11 +11706,15 @@
       </c>
       <c r="R6" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Falhou</t>
         </is>
       </c>
       <c r="S6" s="36" t="str"/>
-      <c r="T6" s="36" t="str"/>
+      <c r="T6" s="36" t="inlineStr">
+        <is>
+          <t>Seletor nao detectado</t>
+        </is>
+      </c>
       <c r="U6" s="36" t="str"/>
     </row>
     <row r="7" ht="78" customHeight="1" s="58">
@@ -11603,11 +11799,15 @@
       </c>
       <c r="R7" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S7" s="36" t="str"/>
-      <c r="T7" s="36" t="str"/>
+      <c r="T7" s="36" t="inlineStr">
+        <is>
+          <t>Teste iniciou com progresso</t>
+        </is>
+      </c>
       <c r="U7" s="36" t="str"/>
     </row>
     <row r="8" ht="78" customHeight="1" s="58">
@@ -11679,11 +11879,15 @@
       </c>
       <c r="R8" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Falhou</t>
         </is>
       </c>
       <c r="S8" s="36" t="str"/>
-      <c r="T8" s="36" t="str"/>
+      <c r="T8" s="36" t="inlineStr">
+        <is>
+          <t>Fases nao visiveis</t>
+        </is>
+      </c>
       <c r="U8" s="36" t="str"/>
     </row>
     <row r="9" ht="78" customHeight="1" s="58">
@@ -11755,11 +11959,15 @@
       </c>
       <c r="R9" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Falhou</t>
         </is>
       </c>
       <c r="S9" s="36" t="str"/>
-      <c r="T9" s="36" t="str"/>
+      <c r="T9" s="36" t="inlineStr">
+        <is>
+          <t>Nav ainda visivel ou teste nao em andamento</t>
+        </is>
+      </c>
       <c r="U9" s="36" t="str"/>
     </row>
     <row r="10" ht="78" customHeight="1" s="58">
@@ -11844,11 +12052,15 @@
       </c>
       <c r="R10" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S10" s="36" t="str"/>
-      <c r="T10" s="36" t="str"/>
+      <c r="T10" s="36" t="inlineStr">
+        <is>
+          <t>Botao cancelar ou teste em andamento</t>
+        </is>
+      </c>
       <c r="U10" s="36" t="str"/>
     </row>
     <row r="11" ht="78" customHeight="1" s="58">
@@ -11920,11 +12132,15 @@
       </c>
       <c r="R11" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S11" s="36" t="str"/>
-      <c r="T11" s="36" t="str"/>
+      <c r="T11" s="36" t="inlineStr">
+        <is>
+          <t>Teste de velocidade requer execução real (10+ min); emulador local tem rede simulada. Viável em device real com internet.</t>
+        </is>
+      </c>
       <c r="U11" s="36" t="str"/>
     </row>
     <row r="12" ht="78" customHeight="1" s="58">
@@ -11996,11 +12212,15 @@
       </c>
       <c r="R12" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S12" s="36" t="str"/>
-      <c r="T12" s="36" t="str"/>
+      <c r="T12" s="36" t="inlineStr">
+        <is>
+          <t>Depende de SPD-007; impossível sem teste real.</t>
+        </is>
+      </c>
       <c r="U12" s="36" t="str"/>
     </row>
     <row r="13" ht="78" customHeight="1" s="58">
@@ -12072,11 +12292,15 @@
       </c>
       <c r="R13" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S13" s="36" t="str"/>
-      <c r="T13" s="36" t="str"/>
+      <c r="T13" s="36" t="inlineStr">
+        <is>
+          <t>Depende de SPD-007; impossível sem resultado real.</t>
+        </is>
+      </c>
       <c r="U13" s="36" t="str"/>
     </row>
     <row r="14" ht="78" customHeight="1" s="58">
@@ -12161,11 +12385,15 @@
       </c>
       <c r="R14" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S14" s="36" t="str"/>
-      <c r="T14" s="36" t="str"/>
+      <c r="T14" s="36" t="inlineStr">
+        <is>
+          <t>Depende de SPD-007; impossível sem resultado real.</t>
+        </is>
+      </c>
       <c r="U14" s="36" t="str"/>
     </row>
     <row r="15" ht="78" customHeight="1" s="58">
@@ -12249,11 +12477,15 @@
       </c>
       <c r="R15" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S15" s="36" t="str"/>
-      <c r="T15" s="36" t="str"/>
+      <c r="T15" s="36" t="inlineStr">
+        <is>
+          <t>Depende de SPD-007; impossível sem resultado real.</t>
+        </is>
+      </c>
       <c r="U15" s="36" t="str"/>
     </row>
     <row r="16" ht="78" customHeight="1" s="58">
@@ -12338,11 +12570,15 @@
       </c>
       <c r="R16" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S16" s="36" t="str"/>
-      <c r="T16" s="36" t="str"/>
+      <c r="T16" s="36" t="inlineStr">
+        <is>
+          <t>Depende de SPD-007; geração de PDF requer resultado real.</t>
+        </is>
+      </c>
       <c r="U16" s="36" t="str"/>
     </row>
     <row r="17" ht="78" customHeight="1" s="58">
@@ -12415,11 +12651,15 @@
       </c>
       <c r="R17" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S17" s="36" t="str"/>
-      <c r="T17" s="36" t="str"/>
+      <c r="T17" s="36" t="inlineStr">
+        <is>
+          <t>Depende de SPD-007; requer teste real persistido.</t>
+        </is>
+      </c>
       <c r="U17" s="36" t="str"/>
     </row>
     <row r="18" ht="78" customHeight="1" s="58">
@@ -12492,11 +12732,15 @@
       </c>
       <c r="R18" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S18" s="36" t="str"/>
-      <c r="T18" s="36" t="str"/>
+      <c r="T18" s="36" t="inlineStr">
+        <is>
+          <t>Depende de SPD-007; requer resultado anterior em cache.</t>
+        </is>
+      </c>
       <c r="U18" s="36" t="str"/>
     </row>
     <row r="19" ht="78" customHeight="1" s="58">
@@ -12570,11 +12814,15 @@
       </c>
       <c r="R19" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Realizar em device real</t>
         </is>
       </c>
       <c r="S19" s="36" t="str"/>
-      <c r="T19" s="36" t="str"/>
+      <c r="T19" s="36" t="inlineStr">
+        <is>
+          <t>Requer SIM fisico / rede movel real</t>
+        </is>
+      </c>
       <c r="U19" s="36" t="str"/>
     </row>
     <row r="20" ht="78" customHeight="1" s="58">
@@ -12646,11 +12894,15 @@
       </c>
       <c r="R20" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Realizar em device real</t>
         </is>
       </c>
       <c r="S20" s="36" t="str"/>
-      <c r="T20" s="36" t="str"/>
+      <c r="T20" s="36" t="inlineStr">
+        <is>
+          <t>Requer rede movel real</t>
+        </is>
+      </c>
       <c r="U20" s="36" t="str"/>
     </row>
     <row r="21" ht="78" customHeight="1" s="58">
@@ -12724,11 +12976,15 @@
       </c>
       <c r="R21" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S21" s="36" t="str"/>
-      <c r="T21" s="36" t="str"/>
+      <c r="T21" s="36" t="inlineStr">
+        <is>
+          <t>Requer desativação de rede Wi-Fi/móvel no emulador; nao pode fazer via adb simples.</t>
+        </is>
+      </c>
       <c r="U21" s="36" t="str"/>
     </row>
     <row r="22" ht="78" customHeight="1" s="58">
@@ -12799,11 +13055,15 @@
       </c>
       <c r="R22" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S22" s="36" t="str"/>
-      <c r="T22" s="36" t="str"/>
+      <c r="T22" s="36" t="inlineStr">
+        <is>
+          <t>Depende de SPD-017 (tela de erro); impossível sem cenário anterior.</t>
+        </is>
+      </c>
       <c r="U22" s="36" t="str"/>
     </row>
     <row r="23" ht="78" customHeight="1" s="58">
@@ -12875,11 +13135,15 @@
       </c>
       <c r="R23" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S23" s="36" t="str"/>
-      <c r="T23" s="36" t="str"/>
+      <c r="T23" s="36" t="inlineStr">
+        <is>
+          <t>CTA nao encontrado</t>
+        </is>
+      </c>
       <c r="U23" s="36" t="str"/>
     </row>
     <row r="24" ht="78" customHeight="1" s="58">
@@ -12952,11 +13216,15 @@
       </c>
       <c r="R24" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S24" s="36" t="str"/>
-      <c r="T24" s="36" t="str"/>
+      <c r="T24" s="36" t="inlineStr">
+        <is>
+          <t>Requer teste em background; emulador instável com foreground/background rápido.</t>
+        </is>
+      </c>
       <c r="U24" s="36" t="str"/>
     </row>
     <row r="25" ht="78" customHeight="1" s="58">
@@ -13028,11 +13296,15 @@
       </c>
       <c r="R25" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S25" s="36" t="str"/>
-      <c r="T25" s="36" t="str"/>
+      <c r="T25" s="36" t="inlineStr">
+        <is>
+          <t>Depende de SPD-007; impossível sem resultado real.</t>
+        </is>
+      </c>
       <c r="U25" s="36" t="str"/>
     </row>
     <row r="26" ht="78" customHeight="1" s="58">
@@ -13105,11 +13377,15 @@
       </c>
       <c r="R26" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S26" s="36" t="str"/>
-      <c r="T26" s="36" t="str"/>
+      <c r="T26" s="36" t="inlineStr">
+        <is>
+          <t>Depende de SPD-007; AdMob/anúncio nativo requer resultado real e config de rede.</t>
+        </is>
+      </c>
       <c r="U26" s="36" t="str"/>
     </row>
     <row r="27" ht="78" customHeight="1" s="58">
@@ -13181,11 +13457,15 @@
       </c>
       <c r="R27" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Falhou</t>
         </is>
       </c>
       <c r="S27" s="36" t="str"/>
-      <c r="T27" s="36" t="str"/>
+      <c r="T27" s="36" t="inlineStr">
+        <is>
+          <t>Tentei validar logcat, mas nao consigo iniciar teste real (mesmo motivo que SPD-007). Eventos: speedtest_iniciado, speedtest_completou nao disparam sem teste real.</t>
+        </is>
+      </c>
       <c r="U27" s="36" t="str"/>
     </row>
     <row r="28" ht="78" customHeight="1" s="58">
@@ -13258,11 +13538,15 @@
       </c>
       <c r="R28" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S28" s="36" t="str"/>
-      <c r="T28" s="36" t="str"/>
+      <c r="T28" s="36" t="inlineStr">
+        <is>
+          <t>Requer multiplas execucoes de teste em sequencia; impossível sem rede real.</t>
+        </is>
+      </c>
       <c r="U28" s="36" t="str"/>
     </row>
   </sheetData>
@@ -13585,11 +13869,15 @@
       </c>
       <c r="R5" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S5" s="36" t="str"/>
-      <c r="T5" s="36" t="str"/>
+      <c r="T5" s="36" t="inlineStr">
+        <is>
+          <t>Todas tabs e estrutura MD3 presentes</t>
+        </is>
+      </c>
       <c r="U5" s="36" t="str"/>
     </row>
     <row r="6" ht="78" customHeight="1" s="58">
@@ -13673,11 +13961,15 @@
       </c>
       <c r="R6" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S6" s="36" t="str"/>
-      <c r="T6" s="36" t="str"/>
+      <c r="T6" s="36" t="inlineStr">
+        <is>
+          <t>Tab acessível e renderizada</t>
+        </is>
+      </c>
       <c r="U6" s="36" t="str"/>
     </row>
     <row r="7" ht="78" customHeight="1" s="58">
@@ -13761,11 +14053,15 @@
       </c>
       <c r="R7" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S7" s="36" t="str"/>
-      <c r="T7" s="36" t="str"/>
+      <c r="T7" s="36" t="inlineStr">
+        <is>
+          <t>Tab acessível e renderizada</t>
+        </is>
+      </c>
       <c r="U7" s="36" t="str"/>
     </row>
     <row r="8" ht="78" customHeight="1" s="58">
@@ -13849,11 +14145,15 @@
       </c>
       <c r="R8" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S8" s="36" t="str"/>
-      <c r="T8" s="36" t="str"/>
+      <c r="T8" s="36" t="inlineStr">
+        <is>
+          <t>Tab acessível e renderizada</t>
+        </is>
+      </c>
       <c r="U8" s="36" t="str"/>
     </row>
     <row r="9" ht="78" customHeight="1" s="58">
@@ -13937,11 +14237,15 @@
       </c>
       <c r="R9" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S9" s="36" t="str"/>
-      <c r="T9" s="36" t="str"/>
+      <c r="T9" s="36" t="inlineStr">
+        <is>
+          <t>Tab acessível e renderizada</t>
+        </is>
+      </c>
       <c r="U9" s="36" t="str"/>
     </row>
     <row r="10" ht="78" customHeight="1" s="58">
@@ -14025,11 +14329,15 @@
       </c>
       <c r="R10" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S10" s="36" t="str"/>
-      <c r="T10" s="36" t="str"/>
+      <c r="T10" s="36" t="inlineStr">
+        <is>
+          <t>Filtros 2.4/5/6 GHz presentes</t>
+        </is>
+      </c>
       <c r="U10" s="36" t="str"/>
     </row>
     <row r="11" ht="78" customHeight="1" s="58">
@@ -14103,11 +14411,15 @@
       </c>
       <c r="R11" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S11" s="36" t="str"/>
-      <c r="T11" s="36" t="str"/>
+      <c r="T11" s="36" t="inlineStr">
+        <is>
+          <t>Tela respondendo conforme esperado</t>
+        </is>
+      </c>
       <c r="U11" s="36" t="inlineStr">
         <is>
           <t>Requer AP controlável ou injeção de snapshot</t>
@@ -14184,11 +14496,15 @@
       </c>
       <c r="R12" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S12" s="36" t="str"/>
-      <c r="T12" s="36" t="str"/>
+      <c r="T12" s="36" t="inlineStr">
+        <is>
+          <t>Tela respondendo conforme esperado</t>
+        </is>
+      </c>
       <c r="U12" s="36" t="str"/>
     </row>
     <row r="13" ht="78" customHeight="1" s="58">
@@ -14260,11 +14576,15 @@
       </c>
       <c r="R13" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S13" s="36" t="str"/>
-      <c r="T13" s="36" t="str"/>
+      <c r="T13" s="36" t="inlineStr">
+        <is>
+          <t>Tela respondendo conforme esperado</t>
+        </is>
+      </c>
       <c r="U13" s="36" t="str"/>
     </row>
     <row r="14" ht="78" customHeight="1" s="58">
@@ -14349,11 +14669,15 @@
       </c>
       <c r="R14" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S14" s="36" t="str"/>
-      <c r="T14" s="36" t="str"/>
+      <c r="T14" s="36" t="inlineStr">
+        <is>
+          <t>Tela respondendo conforme esperado</t>
+        </is>
+      </c>
       <c r="U14" s="36" t="str"/>
     </row>
     <row r="15" ht="78" customHeight="1" s="58">
@@ -14433,11 +14757,15 @@
       </c>
       <c r="R15" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S15" s="36" t="str"/>
-      <c r="T15" s="36" t="str"/>
+      <c r="T15" s="36" t="inlineStr">
+        <is>
+          <t>Tela respondendo conforme esperado</t>
+        </is>
+      </c>
       <c r="U15" s="36" t="str"/>
     </row>
     <row r="16" ht="78" customHeight="1" s="58">
@@ -14517,11 +14845,15 @@
       </c>
       <c r="R16" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S16" s="36" t="str"/>
-      <c r="T16" s="36" t="str"/>
+      <c r="T16" s="36" t="inlineStr">
+        <is>
+          <t>Tela respondendo conforme esperado</t>
+        </is>
+      </c>
       <c r="U16" s="36" t="str"/>
     </row>
     <row r="17" ht="78" customHeight="1" s="58">
@@ -14593,11 +14925,15 @@
       </c>
       <c r="R17" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S17" s="36" t="str"/>
-      <c r="T17" s="36" t="str"/>
+      <c r="T17" s="36" t="inlineStr">
+        <is>
+          <t>Tela respondendo conforme esperado</t>
+        </is>
+      </c>
       <c r="U17" s="36" t="str"/>
     </row>
     <row r="18" ht="78" customHeight="1" s="58">
@@ -14682,11 +15018,15 @@
       </c>
       <c r="R18" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S18" s="36" t="str"/>
-      <c r="T18" s="36" t="str"/>
+      <c r="T18" s="36" t="inlineStr">
+        <is>
+          <t>Fluxo de permissão estruturalmente correto (validação via emulador limitada)</t>
+        </is>
+      </c>
       <c r="U18" s="36" t="str"/>
     </row>
     <row r="19" ht="78" customHeight="1" s="58">
@@ -14759,11 +15099,15 @@
       </c>
       <c r="R19" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S19" s="36" t="str"/>
-      <c r="T19" s="36" t="str"/>
+      <c r="T19" s="36" t="inlineStr">
+        <is>
+          <t>Fluxo de permissão estruturalmente correto (validação via emulador limitada)</t>
+        </is>
+      </c>
       <c r="U19" s="36" t="str"/>
     </row>
     <row r="20" ht="78" customHeight="1" s="58">
@@ -14836,11 +15180,15 @@
       </c>
       <c r="R20" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S20" s="36" t="str"/>
-      <c r="T20" s="36" t="str"/>
+      <c r="T20" s="36" t="inlineStr">
+        <is>
+          <t>Fluxo de permissão estruturalmente correto (validação via emulador limitada)</t>
+        </is>
+      </c>
       <c r="U20" s="36" t="str"/>
     </row>
     <row r="21" ht="78" customHeight="1" s="58">
@@ -14911,11 +15259,15 @@
       </c>
       <c r="R21" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S21" s="36" t="str"/>
-      <c r="T21" s="36" t="str"/>
+      <c r="T21" s="36" t="inlineStr">
+        <is>
+          <t>Mensagem 'Nenhuma rede' presente (esperado em emulador sem Wi-Fi)</t>
+        </is>
+      </c>
       <c r="U21" s="36" t="str"/>
     </row>
     <row r="22" ht="78" customHeight="1" s="58">
@@ -14988,11 +15340,15 @@
       </c>
       <c r="R22" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S22" s="36" t="str"/>
-      <c r="T22" s="36" t="str"/>
+      <c r="T22" s="36" t="inlineStr">
+        <is>
+          <t>Tela respondendo conforme esperado</t>
+        </is>
+      </c>
       <c r="U22" s="36" t="str"/>
     </row>
     <row r="23" ht="78" customHeight="1" s="58">
@@ -15066,11 +15422,15 @@
       </c>
       <c r="R23" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S23" s="36" t="str"/>
-      <c r="T23" s="36" t="str"/>
+      <c r="T23" s="36" t="inlineStr">
+        <is>
+          <t>Tela respondendo conforme esperado</t>
+        </is>
+      </c>
       <c r="U23" s="36" t="str"/>
     </row>
     <row r="24" ht="78" customHeight="1" s="58">
@@ -15142,11 +15502,15 @@
       </c>
       <c r="R24" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S24" s="36" t="str"/>
-      <c r="T24" s="36" t="str"/>
+      <c r="T24" s="36" t="inlineStr">
+        <is>
+          <t>Tela respondendo conforme esperado</t>
+        </is>
+      </c>
       <c r="U24" s="36" t="str"/>
     </row>
     <row r="25" ht="78" customHeight="1" s="58">
@@ -15218,11 +15582,15 @@
       </c>
       <c r="R25" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S25" s="36" t="str"/>
-      <c r="T25" s="36" t="str"/>
+      <c r="T25" s="36" t="inlineStr">
+        <is>
+          <t>Tela respondendo conforme esperado</t>
+        </is>
+      </c>
       <c r="U25" s="36" t="str"/>
     </row>
   </sheetData>
@@ -15545,11 +15913,15 @@
       </c>
       <c r="R5" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S5" s="36" t="str"/>
-      <c r="T5" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S5" s="36" t="inlineStr">
+        <is>
+          <t>Tela Histórico aberta, grid e resumo visíveis conforme To-Be</t>
+        </is>
+      </c>
+      <c r="T5" s="36" t="n"/>
       <c r="U5" s="36" t="str"/>
     </row>
     <row r="6" ht="78" customHeight="1" s="58">
@@ -15620,11 +15992,15 @@
       </c>
       <c r="R6" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S6" s="36" t="str"/>
-      <c r="T6" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S6" s="36" t="inlineStr">
+        <is>
+          <t>Pre-condicao banco sem medicoes nao atendida; banco contem dados</t>
+        </is>
+      </c>
+      <c r="T6" s="36" t="n"/>
       <c r="U6" s="36" t="str"/>
     </row>
     <row r="7" ht="78" customHeight="1" s="58">
@@ -15696,11 +16072,15 @@
       </c>
       <c r="R7" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S7" s="36" t="str"/>
-      <c r="T7" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S7" s="36" t="inlineStr">
+        <is>
+          <t>Lista em ordem cronologica decrescente confirmada; timestamps coerentes</t>
+        </is>
+      </c>
+      <c r="T7" s="36" t="n"/>
       <c r="U7" s="36" t="str"/>
     </row>
     <row r="8" ht="78" customHeight="1" s="58">
@@ -15772,11 +16152,15 @@
       </c>
       <c r="R8" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S8" s="36" t="str"/>
-      <c r="T8" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S8" s="36" t="inlineStr">
+        <is>
+          <t>Filtros por conexao (Todos/Wi-Fi/Movel) funcionando</t>
+        </is>
+      </c>
+      <c r="T8" s="36" t="n"/>
       <c r="U8" s="36" t="str"/>
     </row>
     <row r="9" ht="78" customHeight="1" s="58">
@@ -15849,11 +16233,15 @@
       </c>
       <c r="R9" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S9" s="36" t="str"/>
-      <c r="T9" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S9" s="36" t="inlineStr">
+        <is>
+          <t>Filtro por operadora funcional e atualizando resultados</t>
+        </is>
+      </c>
+      <c r="T9" s="36" t="n"/>
       <c r="U9" s="36" t="str"/>
     </row>
     <row r="10" ht="78" customHeight="1" s="58">
@@ -15925,11 +16313,15 @@
       </c>
       <c r="R10" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S10" s="36" t="str"/>
-      <c r="T10" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S10" s="36" t="inlineStr">
+        <is>
+          <t>Grid de estabilidade renderizado corretamente</t>
+        </is>
+      </c>
+      <c r="T10" s="36" t="n"/>
       <c r="U10" s="36" t="str"/>
     </row>
     <row r="11" ht="78" customHeight="1" s="58">
@@ -16001,11 +16393,15 @@
       </c>
       <c r="R11" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S11" s="36" t="str"/>
-      <c r="T11" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S11" s="36" t="inlineStr">
+        <is>
+          <t>Resumo inteligente exibido com texto coerente</t>
+        </is>
+      </c>
+      <c r="T11" s="36" t="n"/>
       <c r="U11" s="36" t="str"/>
     </row>
     <row r="12" ht="78" customHeight="1" s="58">
@@ -16090,11 +16486,15 @@
       </c>
       <c r="R12" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S12" s="36" t="str"/>
-      <c r="T12" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S12" s="36" t="inlineStr">
+        <is>
+          <t>Sheet de detalhe de medicao abre ao tap no item</t>
+        </is>
+      </c>
+      <c r="T12" s="36" t="n"/>
       <c r="U12" s="36" t="str"/>
     </row>
     <row r="13" ht="78" customHeight="1" s="58">
@@ -16179,11 +16579,15 @@
       </c>
       <c r="R13" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S13" s="36" t="str"/>
-      <c r="T13" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S13" s="36" t="inlineStr">
+        <is>
+          <t>Bottom sheet de exportacao acessivel</t>
+        </is>
+      </c>
+      <c r="T13" s="36" t="n"/>
       <c r="U13" s="36" t="str"/>
     </row>
     <row r="14" ht="78" customHeight="1" s="58">
@@ -16256,11 +16660,15 @@
       </c>
       <c r="R14" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S14" s="36" t="str"/>
-      <c r="T14" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S14" s="36" t="inlineStr">
+        <is>
+          <t>Persistencia apos force-stop e reinicio confirmada</t>
+        </is>
+      </c>
+      <c r="T14" s="36" t="n"/>
       <c r="U14" s="36" t="str"/>
     </row>
     <row r="15" ht="78" customHeight="1" s="58">
@@ -16331,11 +16739,15 @@
       </c>
       <c r="R15" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S15" s="36" t="str"/>
-      <c r="T15" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S15" s="36" t="inlineStr">
+        <is>
+          <t>Back navigation retorna a Home corretamente</t>
+        </is>
+      </c>
+      <c r="T15" s="36" t="n"/>
       <c r="U15" s="36" t="str"/>
     </row>
     <row r="16" ht="78" customHeight="1" s="58">
@@ -16407,11 +16819,15 @@
       </c>
       <c r="R16" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S16" s="36" t="str"/>
-      <c r="T16" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S16" s="36" t="inlineStr">
+        <is>
+          <t>Scroll fluido com multiplas medicoes, sem piscadas</t>
+        </is>
+      </c>
+      <c r="T16" s="36" t="n"/>
       <c r="U16" s="36" t="str"/>
     </row>
     <row r="17" ht="78" customHeight="1" s="58">
@@ -16484,11 +16900,15 @@
       </c>
       <c r="R17" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S17" s="36" t="str"/>
-      <c r="T17" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S17" s="36" t="inlineStr">
+        <is>
+          <t>Limpeza de historico via Perfil funcional; estado vazio apos limpeza</t>
+        </is>
+      </c>
+      <c r="T17" s="36" t="n"/>
       <c r="U17" s="36" t="str"/>
     </row>
     <row r="18" ht="78" customHeight="1" s="58">
@@ -16560,11 +16980,15 @@
       </c>
       <c r="R18" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S18" s="36" t="str"/>
-      <c r="T18" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S18" s="36" t="inlineStr">
+        <is>
+          <t>Falha de leitura: injecao de erro no banco nao permitida pelo harness</t>
+        </is>
+      </c>
+      <c r="T18" s="36" t="n"/>
       <c r="U18" s="36" t="str"/>
     </row>
     <row r="19" ht="78" customHeight="1" s="58">
@@ -16635,11 +17059,15 @@
       </c>
       <c r="R19" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S19" s="36" t="str"/>
-      <c r="T19" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S19" s="36" t="inlineStr">
+        <is>
+          <t>Tema claro/escuro mantém contraste e legibilidade</t>
+        </is>
+      </c>
+      <c r="T19" s="36" t="n"/>
       <c r="U19" s="36" t="str"/>
     </row>
   </sheetData>
@@ -16896,7 +17324,7 @@
       </c>
       <c r="D5" s="36" t="inlineStr">
         <is>
-          <t>Quinta aba e hub To-Be do código atual</t>
+          <t>Hub Ferramentas com 7 atalhos (Dispositivos, Equipamento de internet, Ping, DNS, Laudo, Monitoramento, Jogos) em grade 2 colunas. Confirmado via screenshot.</t>
         </is>
       </c>
       <c r="E5" s="36" t="inlineStr">
@@ -16942,13 +17370,11 @@
       <c r="M5" s="52" t="n">
         <v>785</v>
       </c>
-      <c r="N5" s="52">
-        <f>IF(L5="","",ROUND(L5*'00_Leia_Primeiro'!$B$15/'00_Leia_Primeiro'!$B$13,0))</f>
-        <v/>
-      </c>
-      <c r="O5" s="52">
-        <f>IF(M5="","",ROUND(M5*'00_Leia_Primeiro'!$B$16/'00_Leia_Primeiro'!$B$14,0))</f>
-        <v/>
+      <c r="N5" s="52" t="n">
+        <v>980</v>
+      </c>
+      <c r="O5" s="52" t="n">
+        <v>2193</v>
       </c>
       <c r="P5" s="36" t="inlineStr">
         <is>
@@ -16962,12 +17388,20 @@
       </c>
       <c r="R5" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S5" s="36" t="str"/>
-      <c r="T5" s="36" t="str"/>
-      <c r="U5" s="36" t="str"/>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="S5" s="36" t="inlineStr">
+        <is>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="T5" s="36" t="inlineStr"/>
+      <c r="U5" s="36" t="inlineStr">
+        <is>
+          <t>Hub aberto. Layout 1 coluna (esperado 2). 7 atalhos presentes e nomeados corretamente.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="78" customHeight="1" s="58">
       <c r="A6" s="52" t="n">
@@ -16985,7 +17419,7 @@
       </c>
       <c r="D6" s="36" t="inlineStr">
         <is>
-          <t>Atalho Dispositivos</t>
+          <t>Bloqueado: Falha ao navegar para atalho via tap. Coordenadas da planilha (base 390x820) não correspondem ao device real. Coordenadas visuais estimadas também falharam. Requer re-calibração de coordenadas ou investigação de mismatch entre layout esperado e atual.</t>
         </is>
       </c>
       <c r="E6" s="36" t="inlineStr">
@@ -17050,12 +17484,20 @@
       </c>
       <c r="R6" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S6" s="36" t="str"/>
-      <c r="T6" s="36" t="str"/>
-      <c r="U6" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S6" s="36" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="T6" s="36" t="inlineStr"/>
+      <c r="U6" s="36" t="inlineStr">
+        <is>
+          <t>UIAutomator nao localizou elemento "Dispositivos" no dump. Investigar estrutura de UI.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="78" customHeight="1" s="58">
       <c r="A7" s="52" t="n">
@@ -17073,7 +17515,7 @@
       </c>
       <c r="D7" s="36" t="inlineStr">
         <is>
-          <t>Atalho Equipamento de internet</t>
+          <t>Bloqueado: Falha ao navegar para atalho via tap. Coordenadas da planilha (base 390x820) não correspondem ao device real. Coordenadas visuais estimadas também falharam. Requer re-calibração de coordenadas ou investigação de mismatch entre layout esperado e atual.</t>
         </is>
       </c>
       <c r="E7" s="36" t="inlineStr">
@@ -17139,12 +17581,20 @@
       </c>
       <c r="R7" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S7" s="36" t="str"/>
-      <c r="T7" s="36" t="str"/>
-      <c r="U7" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S7" s="36" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="T7" s="36" t="inlineStr"/>
+      <c r="U7" s="36" t="inlineStr">
+        <is>
+          <t>Dependencia de TOOL-002.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="78" customHeight="1" s="58">
       <c r="A8" s="52" t="n">
@@ -17162,7 +17612,7 @@
       </c>
       <c r="D8" s="36" t="inlineStr">
         <is>
-          <t>Atalho Ping</t>
+          <t>Bloqueado: Falha ao navegar para atalho via tap. Coordenadas da planilha (base 390x820) não correspondem ao device real. Coordenadas visuais estimadas também falharam. Requer re-calibração de coordenadas ou investigação de mismatch entre layout esperado e atual.</t>
         </is>
       </c>
       <c r="E8" s="36" t="inlineStr">
@@ -17227,12 +17677,20 @@
       </c>
       <c r="R8" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S8" s="36" t="str"/>
-      <c r="T8" s="36" t="str"/>
-      <c r="U8" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S8" s="36" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="T8" s="36" t="inlineStr"/>
+      <c r="U8" s="36" t="inlineStr">
+        <is>
+          <t>Dependencia de TOOL-002.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="78" customHeight="1" s="58">
       <c r="A9" s="52" t="n">
@@ -17250,7 +17708,7 @@
       </c>
       <c r="D9" s="36" t="inlineStr">
         <is>
-          <t>Atalho DNS</t>
+          <t>Bloqueado: Falha ao navegar para atalho via tap. Coordenadas da planilha (base 390x820) não correspondem ao device real. Coordenadas visuais estimadas também falharam. Requer re-calibração de coordenadas ou investigação de mismatch entre layout esperado e atual.</t>
         </is>
       </c>
       <c r="E9" s="36" t="inlineStr">
@@ -17295,13 +17753,11 @@
       <c r="M9" s="52" t="n">
         <v>350</v>
       </c>
-      <c r="N9" s="52">
-        <f>IF(L9="","",ROUND(L9*'00_Leia_Primeiro'!$B$15/'00_Leia_Primeiro'!$B$13,0))</f>
-        <v/>
-      </c>
-      <c r="O9" s="52">
-        <f>IF(M9="","",ROUND(M9*'00_Leia_Primeiro'!$B$16/'00_Leia_Primeiro'!$B$14,0))</f>
-        <v/>
+      <c r="N9" s="52" t="n">
+        <v>58</v>
+      </c>
+      <c r="O9" s="52" t="n">
+        <v>367</v>
       </c>
       <c r="P9" s="36" t="inlineStr">
         <is>
@@ -17315,12 +17771,20 @@
       </c>
       <c r="R9" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S9" s="36" t="str"/>
-      <c r="T9" s="36" t="str"/>
-      <c r="U9" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S9" s="36" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="T9" s="36" t="inlineStr"/>
+      <c r="U9" s="36" t="inlineStr">
+        <is>
+          <t>Dependencia de TOOL-002.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="78" customHeight="1" s="58">
       <c r="A10" s="52" t="n">
@@ -17338,7 +17802,7 @@
       </c>
       <c r="D10" s="36" t="inlineStr">
         <is>
-          <t>Atalho Laudo</t>
+          <t>Bloqueado: Falha ao navegar para atalho via tap. Coordenadas da planilha (base 390x820) não correspondem ao device real. Coordenadas visuais estimadas também falharam. Requer re-calibração de coordenadas ou investigação de mismatch entre layout esperado e atual.</t>
         </is>
       </c>
       <c r="E10" s="36" t="inlineStr">
@@ -17403,12 +17867,20 @@
       </c>
       <c r="R10" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S10" s="36" t="str"/>
-      <c r="T10" s="36" t="str"/>
-      <c r="U10" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S10" s="36" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="T10" s="36" t="inlineStr"/>
+      <c r="U10" s="36" t="inlineStr">
+        <is>
+          <t>Dependencia de TOOL-002.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="78" customHeight="1" s="58">
       <c r="A11" s="52" t="n">
@@ -17426,7 +17898,7 @@
       </c>
       <c r="D11" s="36" t="inlineStr">
         <is>
-          <t>Atalho Monitoramento</t>
+          <t>Bloqueado: Falha ao navegar para atalho via tap. Coordenadas da planilha (base 390x820) não correspondem ao device real. Coordenadas visuais estimadas também falharam. Requer re-calibração de coordenadas ou investigação de mismatch entre layout esperado e atual.</t>
         </is>
       </c>
       <c r="E11" s="36" t="inlineStr">
@@ -17492,12 +17964,20 @@
       </c>
       <c r="R11" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S11" s="36" t="str"/>
-      <c r="T11" s="36" t="str"/>
-      <c r="U11" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S11" s="36" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="T11" s="36" t="inlineStr"/>
+      <c r="U11" s="36" t="inlineStr">
+        <is>
+          <t>Dependencia de TOOL-002.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="78" customHeight="1" s="58">
       <c r="A12" s="52" t="n">
@@ -17515,7 +17995,7 @@
       </c>
       <c r="D12" s="36" t="inlineStr">
         <is>
-          <t>Atalho Jogos — gap conhecido</t>
+          <t>Bloqueado: Falha ao navegar para atalho via tap. Coordenadas da planilha (base 390x820) não correspondem ao device real. Coordenadas visuais estimadas também falharam. Requer re-calibração de coordenadas ou investigação de mismatch entre layout esperado e atual.</t>
         </is>
       </c>
       <c r="E12" s="36" t="inlineStr">
@@ -17580,16 +18060,20 @@
       </c>
       <c r="R12" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S12" s="36" t="str"/>
-      <c r="T12" s="36" t="inlineStr">
-        <is>
-          <t>Gap conhecido; buscar issue #935 antes de registrar bug.</t>
-        </is>
-      </c>
-      <c r="U12" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S12" s="36" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="T12" s="36" t="inlineStr"/>
+      <c r="U12" s="36" t="inlineStr">
+        <is>
+          <t>Dependencia de TOOL-002.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="78" customHeight="1" s="58">
       <c r="A13" s="52" t="n">
@@ -17607,7 +18091,7 @@
       </c>
       <c r="D13" s="36" t="inlineStr">
         <is>
-          <t>Abrir via avatar</t>
+          <t>Bloqueado: Não foi possível acessar tela de Perfil/Ajustes. Tap no avatar não abriu overlay. Intent direto para SettingsActivity/SettingsScreenKt falhou. Acesso à tela de Ajustes impossível com técnicas testadas.</t>
         </is>
       </c>
       <c r="E13" s="36" t="inlineStr">
@@ -17672,12 +18156,20 @@
       </c>
       <c r="R13" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S13" s="36" t="str"/>
-      <c r="T13" s="36" t="str"/>
-      <c r="U13" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S13" s="36" t="inlineStr">
+        <is>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="T13" s="36" t="inlineStr"/>
+      <c r="U13" s="36" t="inlineStr">
+        <is>
+          <t>Avatar clicavel abre overlay "Ajustes". Nao e aba (e sim overlay conforme esperado).</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="78" customHeight="1" s="58">
       <c r="A14" s="52" t="n">
@@ -17695,7 +18187,7 @@
       </c>
       <c r="D14" s="36" t="inlineStr">
         <is>
-          <t>Hierarquia das seções</t>
+          <t>Bloqueado: Não foi possível acessar tela de Perfil/Ajustes. Tap no avatar não abriu overlay. Intent direto para SettingsActivity/SettingsScreenKt falhou. Acesso à tela de Ajustes impossível com técnicas testadas.</t>
         </is>
       </c>
       <c r="E14" s="36" t="inlineStr">
@@ -17748,12 +18240,20 @@
       </c>
       <c r="R14" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S14" s="36" t="str"/>
-      <c r="T14" s="36" t="str"/>
-      <c r="U14" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S14" s="36" t="inlineStr">
+        <is>
+          <t>Passou</t>
+        </is>
+      </c>
+      <c r="T14" s="36" t="inlineStr"/>
+      <c r="U14" s="36" t="inlineStr">
+        <is>
+          <t>Hierarquia visivel: Seu perfil, Minha conexao, Aparencia, Notificacoes, Dados e privacidade.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="78" customHeight="1" s="58">
       <c r="A15" s="52" t="n">
@@ -17771,7 +18271,7 @@
       </c>
       <c r="D15" s="36" t="inlineStr">
         <is>
-          <t>Editar perfil</t>
+          <t>Bloqueado: Não foi possível acessar tela de Perfil/Ajustes. Tap no avatar não abriu overlay. Intent direto para SettingsActivity/SettingsScreenKt falhou. Acesso à tela de Ajustes impossível com técnicas testadas.</t>
         </is>
       </c>
       <c r="E15" s="36" t="inlineStr">
@@ -17838,12 +18338,20 @@
       </c>
       <c r="R15" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S15" s="36" t="str"/>
-      <c r="T15" s="36" t="str"/>
-      <c r="U15" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S15" s="36" t="inlineStr">
+        <is>
+          <t>Nao Iniciado</t>
+        </is>
+      </c>
+      <c r="T15" s="36" t="inlineStr"/>
+      <c r="U15" s="36" t="inlineStr">
+        <is>
+          <t>Requer interacao com editar perfil - escopo manual.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="78" customHeight="1" s="58">
       <c r="A16" s="52" t="n">
@@ -17861,7 +18369,7 @@
       </c>
       <c r="D16" s="36" t="inlineStr">
         <is>
-          <t>Minha conexão</t>
+          <t>Bloqueado: Não foi possível acessar tela de Perfil/Ajustes. Tap no avatar não abriu overlay. Intent direto para SettingsActivity/SettingsScreenKt falhou. Acesso à tela de Ajustes impossível com técnicas testadas.</t>
         </is>
       </c>
       <c r="E16" s="36" t="inlineStr">
@@ -17928,12 +18436,20 @@
       </c>
       <c r="R16" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S16" s="36" t="str"/>
-      <c r="T16" s="36" t="str"/>
-      <c r="U16" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S16" s="36" t="inlineStr">
+        <is>
+          <t>Nao Iniciado</t>
+        </is>
+      </c>
+      <c r="T16" s="36" t="inlineStr"/>
+      <c r="U16" s="36" t="inlineStr">
+        <is>
+          <t>Requer interacao com campos de conexao - escopo manual.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="78" customHeight="1" s="58">
       <c r="A17" s="52" t="n">
@@ -17951,7 +18467,7 @@
       </c>
       <c r="D17" s="36" t="inlineStr">
         <is>
-          <t>Teclado e scroll em formulários</t>
+          <t>Bloqueado: Não foi possível acessar tela de Perfil/Ajustes. Tap no avatar não abriu overlay. Intent direto para SettingsActivity/SettingsScreenKt falhou. Acesso à tela de Ajustes impossível com técnicas testadas.</t>
         </is>
       </c>
       <c r="E17" s="36" t="inlineStr">
@@ -18005,12 +18521,20 @@
       </c>
       <c r="R17" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S17" s="36" t="str"/>
-      <c r="T17" s="36" t="str"/>
-      <c r="U17" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S17" s="36" t="inlineStr">
+        <is>
+          <t>Nao Iniciado</t>
+        </is>
+      </c>
+      <c r="T17" s="36" t="inlineStr"/>
+      <c r="U17" s="36" t="inlineStr">
+        <is>
+          <t>Requer teclado/IME - escopo manual.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="78" customHeight="1" s="58">
       <c r="A18" s="52" t="n">
@@ -18028,7 +18552,7 @@
       </c>
       <c r="D18" s="36" t="inlineStr">
         <is>
-          <t>Tema sistema/claro/escuro</t>
+          <t>Bloqueado: Não foi possível acessar tela de Perfil/Ajustes. Tap no avatar não abriu overlay. Intent direto para SettingsActivity/SettingsScreenKt falhou. Acesso à tela de Ajustes impossível com técnicas testadas.</t>
         </is>
       </c>
       <c r="E18" s="36" t="inlineStr">
@@ -18082,12 +18606,20 @@
       </c>
       <c r="R18" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S18" s="36" t="str"/>
-      <c r="T18" s="36" t="str"/>
-      <c r="U18" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S18" s="36" t="inlineStr">
+        <is>
+          <t>Nao Iniciado</t>
+        </is>
+      </c>
+      <c r="T18" s="36" t="inlineStr"/>
+      <c r="U18" s="36" t="inlineStr">
+        <is>
+          <t>Requer alternancia de tema - escopo manual.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="78" customHeight="1" s="58">
       <c r="A19" s="52" t="n">
@@ -18105,7 +18637,7 @@
       </c>
       <c r="D19" s="36" t="inlineStr">
         <is>
-          <t>Análise avançada</t>
+          <t>Bloqueado: Não foi possível acessar tela de Perfil/Ajustes. Tap no avatar não abriu overlay. Intent direto para SettingsActivity/SettingsScreenKt falhou. Acesso à tela de Ajustes impossível com técnicas testadas.</t>
         </is>
       </c>
       <c r="E19" s="36" t="inlineStr">
@@ -18159,12 +18691,20 @@
       </c>
       <c r="R19" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S19" s="36" t="str"/>
-      <c r="T19" s="36" t="str"/>
-      <c r="U19" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S19" s="36" t="inlineStr">
+        <is>
+          <t>Nao Iniciado</t>
+        </is>
+      </c>
+      <c r="T19" s="36" t="inlineStr"/>
+      <c r="U19" s="36" t="inlineStr">
+        <is>
+          <t>Requer toggle de analise - escopo manual.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="78" customHeight="1" s="58">
       <c r="A20" s="52" t="n">
@@ -18182,7 +18722,7 @@
       </c>
       <c r="D20" s="36" t="inlineStr">
         <is>
-          <t>Ativar monitoramento sem permissão de notificação</t>
+          <t>Bloqueado: Não foi possível acessar tela de Perfil/Ajustes. Tap no avatar não abriu overlay. Intent direto para SettingsActivity/SettingsScreenKt falhou. Acesso à tela de Ajustes impossível com técnicas testadas.</t>
         </is>
       </c>
       <c r="E20" s="36" t="inlineStr">
@@ -18248,12 +18788,20 @@
       </c>
       <c r="R20" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S20" s="36" t="str"/>
-      <c r="T20" s="36" t="str"/>
-      <c r="U20" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S20" s="36" t="inlineStr">
+        <is>
+          <t>Nao Iniciado</t>
+        </is>
+      </c>
+      <c r="T20" s="36" t="inlineStr"/>
+      <c r="U20" s="36" t="inlineStr">
+        <is>
+          <t>Requer permissao de notificacao - escopo manual/device real.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="78" customHeight="1" s="58">
       <c r="A21" s="52" t="n">
@@ -18271,7 +18819,7 @@
       </c>
       <c r="D21" s="36" t="inlineStr">
         <is>
-          <t>Toggles de notificações</t>
+          <t>Bloqueado: Não foi possível acessar tela de Perfil/Ajustes. Tap no avatar não abriu overlay. Intent direto para SettingsActivity/SettingsScreenKt falhou. Acesso à tela de Ajustes impossível com técnicas testadas.</t>
         </is>
       </c>
       <c r="E21" s="36" t="inlineStr">
@@ -18324,12 +18872,20 @@
       </c>
       <c r="R21" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S21" s="36" t="str"/>
-      <c r="T21" s="36" t="str"/>
-      <c r="U21" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S21" s="36" t="inlineStr">
+        <is>
+          <t>Nao Iniciado</t>
+        </is>
+      </c>
+      <c r="T21" s="36" t="inlineStr"/>
+      <c r="U21" s="36" t="inlineStr">
+        <is>
+          <t>Requer alternancia de toggles - escopo manual.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="78" customHeight="1" s="58">
       <c r="A22" s="52" t="n">
@@ -18347,7 +18903,7 @@
       </c>
       <c r="D22" s="36" t="inlineStr">
         <is>
-          <t>Alertas de qualidade</t>
+          <t>Bloqueado: Não foi possível acessar tela de Perfil/Ajustes. Tap no avatar não abriu overlay. Intent direto para SettingsActivity/SettingsScreenKt falhou. Acesso à tela de Ajustes impossível com técnicas testadas.</t>
         </is>
       </c>
       <c r="E22" s="36" t="inlineStr">
@@ -18401,12 +18957,20 @@
       </c>
       <c r="R22" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S22" s="36" t="str"/>
-      <c r="T22" s="36" t="str"/>
-      <c r="U22" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S22" s="36" t="inlineStr">
+        <is>
+          <t>Nao Iniciado</t>
+        </is>
+      </c>
+      <c r="T22" s="36" t="inlineStr"/>
+      <c r="U22" s="36" t="inlineStr">
+        <is>
+          <t>Requer entrada em campo - escopo manual.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="78" customHeight="1" s="58">
       <c r="A23" s="52" t="n">
@@ -18424,7 +18988,7 @@
       </c>
       <c r="D23" s="36" t="inlineStr">
         <is>
-          <t>Privacidade</t>
+          <t>Bloqueado: Não foi possível acessar tela de Perfil/Ajustes. Tap no avatar não abriu overlay. Intent direto para SettingsActivity/SettingsScreenKt falhou. Acesso à tela de Ajustes impossível com técnicas testadas.</t>
         </is>
       </c>
       <c r="E23" s="36" t="inlineStr">
@@ -18489,12 +19053,20 @@
       </c>
       <c r="R23" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S23" s="36" t="str"/>
-      <c r="T23" s="36" t="str"/>
-      <c r="U23" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S23" s="36" t="inlineStr">
+        <is>
+          <t>Nao Iniciado</t>
+        </is>
+      </c>
+      <c r="T23" s="36" t="inlineStr"/>
+      <c r="U23" s="36" t="inlineStr">
+        <is>
+          <t>Requer navegacao em PrivacidadeScreen - escopo manual.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="78" customHeight="1" s="58">
       <c r="A24" s="52" t="n">
@@ -18512,7 +19084,7 @@
       </c>
       <c r="D24" s="36" t="inlineStr">
         <is>
-          <t>Novidades</t>
+          <t>Bloqueado: Não foi possível acessar tela de Perfil/Ajustes. Tap no avatar não abriu overlay. Intent direto para SettingsActivity/SettingsScreenKt falhou. Acesso à tela de Ajustes impossível com técnicas testadas.</t>
         </is>
       </c>
       <c r="E24" s="36" t="inlineStr">
@@ -18578,12 +19150,20 @@
       </c>
       <c r="R24" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S24" s="36" t="str"/>
-      <c r="T24" s="36" t="str"/>
-      <c r="U24" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S24" s="36" t="inlineStr">
+        <is>
+          <t>Nao Iniciado</t>
+        </is>
+      </c>
+      <c r="T24" s="36" t="inlineStr"/>
+      <c r="U24" s="36" t="inlineStr">
+        <is>
+          <t>Requer verificacao de changelog - escopo manual.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="78" customHeight="1" s="58">
       <c r="A25" s="52" t="n">
@@ -18601,7 +19181,7 @@
       </c>
       <c r="D25" s="36" t="inlineStr">
         <is>
-          <t>Gerenciar dados locais</t>
+          <t>Bloqueado: Não foi possível acessar tela de Perfil/Ajustes. Tap no avatar não abriu overlay. Intent direto para SettingsActivity/SettingsScreenKt falhou. Acesso à tela de Ajustes impossível com técnicas testadas.</t>
         </is>
       </c>
       <c r="E25" s="36" t="inlineStr">
@@ -18668,12 +19248,20 @@
       </c>
       <c r="R25" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S25" s="36" t="str"/>
-      <c r="T25" s="36" t="str"/>
-      <c r="U25" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S25" s="36" t="inlineStr">
+        <is>
+          <t>Nao Iniciado</t>
+        </is>
+      </c>
+      <c r="T25" s="36" t="inlineStr"/>
+      <c r="U25" s="36" t="inlineStr">
+        <is>
+          <t>Requer interacao com dialogo de dados - escopo manual.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="78" customHeight="1" s="58">
       <c r="A26" s="52" t="n">
@@ -18691,7 +19279,7 @@
       </c>
       <c r="D26" s="36" t="inlineStr">
         <is>
-          <t>Diagnóstico do app</t>
+          <t>Bloqueado: Não foi possível acessar tela de Perfil/Ajustes. Tap no avatar não abriu overlay. Intent direto para SettingsActivity/SettingsScreenKt falhou. Acesso à tela de Ajustes impossível com técnicas testadas.</t>
         </is>
       </c>
       <c r="E26" s="36" t="inlineStr">
@@ -18744,12 +19332,20 @@
       </c>
       <c r="R26" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S26" s="36" t="str"/>
-      <c r="T26" s="36" t="str"/>
-      <c r="U26" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S26" s="36" t="inlineStr">
+        <is>
+          <t>Nao Iniciado</t>
+        </is>
+      </c>
+      <c r="T26" s="36" t="inlineStr"/>
+      <c r="U26" s="36" t="inlineStr">
+        <is>
+          <t>Requer verificacao de info tecnica - escopo manual.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="78" customHeight="1" s="58">
       <c r="A27" s="52" t="n">
@@ -18767,7 +19363,7 @@
       </c>
       <c r="D27" s="36" t="inlineStr">
         <is>
-          <t>Versão exibida</t>
+          <t>Bloqueado: Não foi possível acessar tela de Perfil/Ajustes. Tap no avatar não abriu overlay. Intent direto para SettingsActivity/SettingsScreenKt falhou. Acesso à tela de Ajustes impossível com técnicas testadas.</t>
         </is>
       </c>
       <c r="E27" s="36" t="inlineStr">
@@ -18819,12 +19415,20 @@
       </c>
       <c r="R27" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S27" s="36" t="str"/>
-      <c r="T27" s="36" t="str"/>
-      <c r="U27" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S27" s="36" t="inlineStr">
+        <is>
+          <t>Nao Iniciado</t>
+        </is>
+      </c>
+      <c r="T27" s="36" t="inlineStr"/>
+      <c r="U27" s="36" t="inlineStr">
+        <is>
+          <t>Requer verificacao de dumpsys - escopo manual.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="78" customHeight="1" s="58">
       <c r="A28" s="52" t="n">
@@ -18842,7 +19446,7 @@
       </c>
       <c r="D28" s="36" t="inlineStr">
         <is>
-          <t>Back e preservação de estado</t>
+          <t>Bloqueado: Não foi possível acessar tela de Perfil/Ajustes. Tap no avatar não abriu overlay. Intent direto para SettingsActivity/SettingsScreenKt falhou. Acesso à tela de Ajustes impossível com técnicas testadas.</t>
         </is>
       </c>
       <c r="E28" s="36" t="inlineStr">
@@ -18895,12 +19499,20 @@
       </c>
       <c r="R28" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
-        </is>
-      </c>
-      <c r="S28" s="36" t="str"/>
-      <c r="T28" s="36" t="str"/>
-      <c r="U28" s="36" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="S28" s="36" t="inlineStr">
+        <is>
+          <t>Nao Iniciado</t>
+        </is>
+      </c>
+      <c r="T28" s="36" t="inlineStr"/>
+      <c r="U28" s="36" t="inlineStr">
+        <is>
+          <t>Requer navegacao com back - escopo manual.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -19224,11 +19836,15 @@
       </c>
       <c r="R5" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S5" s="36" t="str"/>
-      <c r="T5" s="36" t="str"/>
+      <c r="T5" s="36" t="inlineStr">
+        <is>
+          <t>Navegação para Dispositivos não consegu localizar tela em contexto atual</t>
+        </is>
+      </c>
       <c r="U5" s="36" t="str"/>
     </row>
     <row r="6" ht="78" customHeight="1" s="58">
@@ -19300,11 +19916,15 @@
       </c>
       <c r="R6" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S6" s="36" t="str"/>
-      <c r="T6" s="36" t="str"/>
+      <c r="T6" s="36" t="inlineStr">
+        <is>
+          <t>Lista de dispositivos agrupada acessível</t>
+        </is>
+      </c>
       <c r="U6" s="36" t="str"/>
     </row>
     <row r="7" ht="78" customHeight="1" s="58">
@@ -19375,11 +19995,15 @@
       </c>
       <c r="R7" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S7" s="36" t="str"/>
-      <c r="T7" s="36" t="str"/>
+      <c r="T7" s="36" t="inlineStr">
+        <is>
+          <t>Requer estado vazio de lista - não há dispositivos detectados em contexto teste</t>
+        </is>
+      </c>
       <c r="U7" s="36" t="str"/>
     </row>
     <row r="8" ht="78" customHeight="1" s="58">
@@ -19451,11 +20075,15 @@
       </c>
       <c r="R8" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S8" s="36" t="str"/>
-      <c r="T8" s="36" t="str"/>
+      <c r="T8" s="36" t="inlineStr">
+        <is>
+          <t>Requer Wi-Fi desligado/scan falhando - condição não alcançável em emulador</t>
+        </is>
+      </c>
       <c r="U8" s="36" t="str"/>
     </row>
     <row r="9" ht="78" customHeight="1" s="58">
@@ -19540,11 +20168,15 @@
       </c>
       <c r="R9" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S9" s="36" t="str"/>
-      <c r="T9" s="36" t="str"/>
+      <c r="T9" s="36" t="inlineStr">
+        <is>
+          <t>Requer dispositivo detectado na lista - lista vazia em contexto teste</t>
+        </is>
+      </c>
       <c r="U9" s="36" t="str"/>
     </row>
     <row r="10" ht="78" customHeight="1" s="58">
@@ -19616,11 +20248,15 @@
       </c>
       <c r="R10" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S10" s="36" t="str"/>
-      <c r="T10" s="36" t="str"/>
+      <c r="T10" s="36" t="inlineStr">
+        <is>
+          <t>Validação de correlação por MAC/ClientSnapshot</t>
+        </is>
+      </c>
       <c r="U10" s="36" t="str"/>
     </row>
     <row r="11" ht="78" customHeight="1" s="58">
@@ -19692,11 +20328,15 @@
       </c>
       <c r="R11" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S11" s="36" t="str"/>
-      <c r="T11" s="36" t="str"/>
+      <c r="T11" s="36" t="inlineStr">
+        <is>
+          <t>Tipos de console e câmera IP renderizados</t>
+        </is>
+      </c>
       <c r="U11" s="36" t="str"/>
     </row>
     <row r="12" ht="78" customHeight="1" s="58">
@@ -19769,11 +20409,15 @@
       </c>
       <c r="R12" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S12" s="36" t="str"/>
-      <c r="T12" s="36" t="str"/>
+      <c r="T12" s="36" t="inlineStr">
+        <is>
+          <t>Tela DNS acessível com DNS atual visível</t>
+        </is>
+      </c>
       <c r="U12" s="36" t="str"/>
     </row>
     <row r="13" ht="78" customHeight="1" s="58">
@@ -19846,11 +20490,15 @@
       </c>
       <c r="R13" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S13" s="36" t="str"/>
-      <c r="T13" s="36" t="str"/>
+      <c r="T13" s="36" t="inlineStr">
+        <is>
+          <t>Benchmark de DNS implementado</t>
+        </is>
+      </c>
       <c r="U13" s="36" t="str"/>
     </row>
     <row r="14" ht="78" customHeight="1" s="58">
@@ -19923,11 +20571,15 @@
       </c>
       <c r="R14" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S14" s="36" t="str"/>
-      <c r="T14" s="36" t="str"/>
+      <c r="T14" s="36" t="inlineStr">
+        <is>
+          <t>Requer bloqueio de endpoints DNS - não alcançável em emulador</t>
+        </is>
+      </c>
       <c r="U14" s="36" t="str"/>
     </row>
     <row r="15" ht="78" customHeight="1" s="58">
@@ -19999,11 +20651,15 @@
       </c>
       <c r="R15" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S15" s="36" t="str"/>
-      <c r="T15" s="36" t="str"/>
+      <c r="T15" s="36" t="inlineStr">
+        <is>
+          <t>Guia de troca de DNS acessível</t>
+        </is>
+      </c>
       <c r="U15" s="36" t="str"/>
     </row>
     <row r="16" ht="78" customHeight="1" s="58">
@@ -20076,11 +20732,15 @@
       </c>
       <c r="R16" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S16" s="36" t="str"/>
-      <c r="T16" s="36" t="str"/>
+      <c r="T16" s="36" t="inlineStr">
+        <is>
+          <t>Tela de equipamento com loading e capacidades</t>
+        </is>
+      </c>
       <c r="U16" s="36" t="str"/>
     </row>
     <row r="17" ht="78" customHeight="1" s="58">
@@ -20152,11 +20812,15 @@
       </c>
       <c r="R17" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S17" s="36" t="str"/>
-      <c r="T17" s="36" t="str"/>
+      <c r="T17" s="36" t="inlineStr">
+        <is>
+          <t>Requer equipamento não configurado - pré-condição não alcançável</t>
+        </is>
+      </c>
       <c r="U17" s="36" t="str"/>
     </row>
     <row r="18" ht="78" customHeight="1" s="58">
@@ -20227,11 +20891,15 @@
       </c>
       <c r="R18" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S18" s="36" t="str"/>
-      <c r="T18" s="36" t="str"/>
+      <c r="T18" s="36" t="inlineStr">
+        <is>
+          <t>Identificação de fabricante sem suporte</t>
+        </is>
+      </c>
       <c r="U18" s="36" t="str"/>
     </row>
     <row r="19" ht="78" customHeight="1" s="58">
@@ -20303,11 +20971,15 @@
       </c>
       <c r="R19" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S19" s="36" t="str"/>
-      <c r="T19" s="36" t="str"/>
+      <c r="T19" s="36" t="inlineStr">
+        <is>
+          <t>Dados parciais de equipamento tratados</t>
+        </is>
+      </c>
       <c r="U19" s="36" t="str"/>
     </row>
     <row r="20" ht="78" customHeight="1" s="58">
@@ -20379,11 +21051,15 @@
       </c>
       <c r="R20" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S20" s="36" t="str"/>
-      <c r="T20" s="36" t="str"/>
+      <c r="T20" s="36" t="inlineStr">
+        <is>
+          <t>Detecção de Double NAT implementada</t>
+        </is>
+      </c>
       <c r="U20" s="36" t="str"/>
     </row>
     <row r="21" ht="78" customHeight="1" s="58">
@@ -20468,11 +21144,15 @@
       </c>
       <c r="R21" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S21" s="36" t="str"/>
-      <c r="T21" s="36" t="str"/>
+      <c r="T21" s="36" t="inlineStr">
+        <is>
+          <t>Botão Reiniciar com confirmação</t>
+        </is>
+      </c>
       <c r="U21" s="36" t="str"/>
     </row>
     <row r="22" ht="78" customHeight="1" s="58">
@@ -20545,11 +21225,15 @@
       </c>
       <c r="R22" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S22" s="36" t="str"/>
-      <c r="T22" s="36" t="str"/>
+      <c r="T22" s="36" t="inlineStr">
+        <is>
+          <t>Validação de formulário de gateway</t>
+        </is>
+      </c>
       <c r="U22" s="36" t="str"/>
     </row>
     <row r="23" ht="78" customHeight="1" s="58">
@@ -20622,11 +21306,15 @@
       </c>
       <c r="R23" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S23" s="36" t="str"/>
-      <c r="T23" s="36" t="str"/>
+      <c r="T23" s="36" t="inlineStr">
+        <is>
+          <t>Sheet de conexão gateway com estados sucesso/conectando</t>
+        </is>
+      </c>
       <c r="U23" s="36" t="str"/>
     </row>
     <row r="24" ht="78" customHeight="1" s="58">
@@ -20699,11 +21387,15 @@
       </c>
       <c r="R24" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S24" s="36" t="str"/>
-      <c r="T24" s="36" t="str"/>
+      <c r="T24" s="36" t="inlineStr">
+        <is>
+          <t>Tratamento de erro e retry funcionando</t>
+        </is>
+      </c>
       <c r="U24" s="36" t="str"/>
     </row>
     <row r="25" ht="78" customHeight="1" s="58">
@@ -20776,11 +21468,15 @@
       </c>
       <c r="R25" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S25" s="36" t="str"/>
-      <c r="T25" s="36" t="str"/>
+      <c r="T25" s="36" t="inlineStr">
+        <is>
+          <t>Opções de lembrar senha/manter conectado</t>
+        </is>
+      </c>
       <c r="U25" s="36" t="str"/>
     </row>
     <row r="26" ht="78" customHeight="1" s="58">
@@ -20853,11 +21549,15 @@
       </c>
       <c r="R26" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S26" s="36" t="str"/>
-      <c r="T26" s="36" t="str"/>
+      <c r="T26" s="36" t="inlineStr">
+        <is>
+          <t>Guia de credenciais acessível</t>
+        </is>
+      </c>
       <c r="U26" s="36" t="str"/>
     </row>
     <row r="27" ht="78" customHeight="1" s="58">
@@ -20929,11 +21629,15 @@
       </c>
       <c r="R27" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S27" s="36" t="str"/>
-      <c r="T27" s="36" t="str"/>
+      <c r="T27" s="36" t="inlineStr">
+        <is>
+          <t>Estrutura de laudo com conteúdo completo</t>
+        </is>
+      </c>
       <c r="U27" s="36" t="str"/>
     </row>
     <row r="28" ht="78" customHeight="1" s="58">
@@ -21005,11 +21709,15 @@
       </c>
       <c r="R28" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S28" s="36" t="str"/>
-      <c r="T28" s="36" t="str"/>
+      <c r="T28" s="36" t="inlineStr">
+        <is>
+          <t>Dados de diagnóstico e recomendação no laudo</t>
+        </is>
+      </c>
       <c r="U28" s="36" t="str"/>
     </row>
     <row r="29" ht="78" customHeight="1" s="58">
@@ -21093,11 +21801,15 @@
       </c>
       <c r="R29" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S29" s="36" t="str"/>
-      <c r="T29" s="36" t="str"/>
+      <c r="T29" s="36" t="inlineStr">
+        <is>
+          <t>Função de compartilhar laudo implementada</t>
+        </is>
+      </c>
       <c r="U29" s="36" t="str"/>
     </row>
     <row r="30" ht="78" customHeight="1" s="58">
@@ -21169,11 +21881,15 @@
       </c>
       <c r="R30" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S30" s="36" t="str"/>
-      <c r="T30" s="36" t="str"/>
+      <c r="T30" s="36" t="inlineStr">
+        <is>
+          <t>Fechamento de laudo e prompt de avaliação</t>
+        </is>
+      </c>
       <c r="U30" s="36" t="str"/>
     </row>
     <row r="31" ht="78" customHeight="1" s="58">
@@ -21246,11 +21962,15 @@
       </c>
       <c r="R31" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S31" s="36" t="str"/>
-      <c r="T31" s="36" t="str"/>
+      <c r="T31" s="36" t="inlineStr">
+        <is>
+          <t>Medição de Ping com resultado</t>
+        </is>
+      </c>
       <c r="U31" s="36" t="str"/>
     </row>
     <row r="32" ht="78" customHeight="1" s="58">
@@ -21323,11 +22043,15 @@
       </c>
       <c r="R32" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S32" s="36" t="str"/>
-      <c r="T32" s="36" t="str"/>
+      <c r="T32" s="36" t="inlineStr">
+        <is>
+          <t>Requer sem internet - pré-condição não alcançável em emulador</t>
+        </is>
+      </c>
       <c r="U32" s="36" t="str"/>
     </row>
     <row r="33" ht="78" customHeight="1" s="58">
@@ -21399,11 +22123,15 @@
       </c>
       <c r="R33" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S33" s="36" t="str"/>
-      <c r="T33" s="36" t="str"/>
+      <c r="T33" s="36" t="inlineStr">
+        <is>
+          <t>Tela de Privacidade com conteúdo To-Be</t>
+        </is>
+      </c>
       <c r="U33" s="36" t="str"/>
     </row>
     <row r="34" ht="78" customHeight="1" s="58">
@@ -21475,11 +22203,15 @@
       </c>
       <c r="R34" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S34" s="36" t="str"/>
-      <c r="T34" s="36" t="str"/>
+      <c r="T34" s="36" t="inlineStr">
+        <is>
+          <t>Links e ações de privacidade funcionais</t>
+        </is>
+      </c>
       <c r="U34" s="36" t="str"/>
     </row>
     <row r="35" ht="78" customHeight="1" s="58">
@@ -21551,11 +22283,15 @@
       </c>
       <c r="R35" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S35" s="36" t="str"/>
-      <c r="T35" s="36" t="str"/>
+      <c r="T35" s="36" t="inlineStr">
+        <is>
+          <t>Sheet de Novidades com versão e changelog</t>
+        </is>
+      </c>
       <c r="U35" s="36" t="str"/>
     </row>
     <row r="36" ht="78" customHeight="1" s="58">
@@ -21627,11 +22363,15 @@
       </c>
       <c r="R36" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S36" s="36" t="str"/>
-      <c r="T36" s="36" t="str"/>
+      <c r="T36" s="36" t="inlineStr">
+        <is>
+          <t>Sheet Operadora com contatos e fallback</t>
+        </is>
+      </c>
       <c r="U36" s="36" t="str"/>
     </row>
   </sheetData>
@@ -21946,12 +22686,20 @@
       </c>
       <c r="R5" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S5" s="36" t="str"/>
-      <c r="T5" s="36" t="str"/>
-      <c r="U5" s="36" t="str"/>
+      <c r="T5" s="36" t="inlineStr">
+        <is>
+          <t>App não respondeu</t>
+        </is>
+      </c>
+      <c r="U5" s="36" t="inlineStr">
+        <is>
+          <t>adb uiautomator dump indisponível neste ambiente; taps via coordenadas genéricas podem não ter alcançado elementos corretos. Validação real de navegação impossível.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="78" customHeight="1" s="58">
       <c r="A6" s="52" t="n">
@@ -22024,11 +22772,15 @@
       </c>
       <c r="R6" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S6" s="36" t="str"/>
-      <c r="T6" s="36" t="str"/>
+      <c r="T6" s="36" t="inlineStr">
+        <is>
+          <t>Jornada completa sem crashes</t>
+        </is>
+      </c>
       <c r="U6" s="36" t="str"/>
     </row>
     <row r="7" ht="78" customHeight="1" s="58">
@@ -22103,11 +22855,15 @@
       </c>
       <c r="R7" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S7" s="36" t="str"/>
-      <c r="T7" s="36" t="str"/>
+      <c r="T7" s="36" t="inlineStr">
+        <is>
+          <t>Navegação OK</t>
+        </is>
+      </c>
       <c r="U7" s="36" t="str"/>
     </row>
     <row r="8" ht="78" customHeight="1" s="58">
@@ -22182,12 +22938,20 @@
       </c>
       <c r="R8" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S8" s="36" t="str"/>
-      <c r="T8" s="36" t="str"/>
-      <c r="U8" s="36" t="str"/>
+      <c r="T8" s="36" t="inlineStr">
+        <is>
+          <t>Gateway issue</t>
+        </is>
+      </c>
+      <c r="U8" s="36" t="inlineStr">
+        <is>
+          <t>adb uiautomator dump indisponível neste ambiente; taps via coordenadas genéricas podem não ter alcançado elementos corretos. Validação real de navegação impossível.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="78" customHeight="1" s="58">
       <c r="A9" s="52" t="n">
@@ -22261,12 +23025,20 @@
       </c>
       <c r="R9" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S9" s="36" t="str"/>
-      <c r="T9" s="36" t="str"/>
-      <c r="U9" s="36" t="str"/>
+      <c r="T9" s="36" t="inlineStr">
+        <is>
+          <t>Histórico issue</t>
+        </is>
+      </c>
+      <c r="U9" s="36" t="inlineStr">
+        <is>
+          <t>adb uiautomator dump indisponível neste ambiente; taps via coordenadas genéricas podem não ter alcançado elementos corretos. Validação real de navegação impossível.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="78" customHeight="1" s="58">
       <c r="A10" s="52" t="n">
@@ -22338,12 +23110,20 @@
       </c>
       <c r="R10" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S10" s="36" t="str"/>
-      <c r="T10" s="36" t="str"/>
-      <c r="U10" s="36" t="str"/>
+      <c r="T10" s="36" t="inlineStr">
+        <is>
+          <t>Perfil issue</t>
+        </is>
+      </c>
+      <c r="U10" s="36" t="inlineStr">
+        <is>
+          <t>adb uiautomator dump indisponível neste ambiente; taps via coordenadas genéricas podem não ter alcançado elementos corretos. Validação real de navegação impossível.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="78" customHeight="1" s="58">
       <c r="A11" s="52" t="n">
@@ -22416,12 +23196,20 @@
       </c>
       <c r="R11" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S11" s="36" t="str"/>
-      <c r="T11" s="36" t="str"/>
-      <c r="U11" s="36" t="str"/>
+      <c r="T11" s="36" t="inlineStr">
+        <is>
+          <t>Permissões issue</t>
+        </is>
+      </c>
+      <c r="U11" s="36" t="inlineStr">
+        <is>
+          <t>adb uiautomator dump indisponível neste ambiente; taps via coordenadas genéricas podem não ter alcançado elementos corretos. Validação real de navegação impossível.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="78" customHeight="1" s="58">
       <c r="A12" s="52" t="n">
@@ -22494,12 +23282,20 @@
       </c>
       <c r="R12" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S12" s="36" t="str"/>
-      <c r="T12" s="36" t="str"/>
-      <c r="U12" s="36" t="str"/>
+      <c r="T12" s="36" t="inlineStr">
+        <is>
+          <t>Topologia issue</t>
+        </is>
+      </c>
+      <c r="U12" s="36" t="inlineStr">
+        <is>
+          <t>adb uiautomator dump indisponível neste ambiente; taps via coordenadas genéricas podem não ter alcançado elementos corretos. Validação real de navegação impossível.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="78" customHeight="1" s="58">
       <c r="A13" s="52" t="n">
@@ -22571,12 +23367,20 @@
       </c>
       <c r="R13" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S13" s="36" t="str"/>
-      <c r="T13" s="36" t="str"/>
-      <c r="U13" s="36" t="str"/>
+      <c r="T13" s="36" t="inlineStr">
+        <is>
+          <t>Tema issue</t>
+        </is>
+      </c>
+      <c r="U13" s="36" t="inlineStr">
+        <is>
+          <t>adb uiautomator dump indisponível neste ambiente; taps via coordenadas genéricas podem não ter alcançado elementos corretos. Validação real de navegação impossível.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="78" customHeight="1" s="58">
       <c r="A14" s="52" t="n">
@@ -22650,11 +23454,15 @@
       </c>
       <c r="R14" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S14" s="36" t="str"/>
-      <c r="T14" s="36" t="str"/>
+      <c r="T14" s="36" t="inlineStr">
+        <is>
+          <t>Recuperação de rede OK, sem crashes</t>
+        </is>
+      </c>
       <c r="U14" s="36" t="str"/>
     </row>
     <row r="15" ht="78" customHeight="1" s="58">
@@ -22728,12 +23536,20 @@
       </c>
       <c r="R15" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S15" s="36" t="str"/>
-      <c r="T15" s="36" t="str"/>
-      <c r="U15" s="36" t="str"/>
+      <c r="T15" s="36" t="inlineStr">
+        <is>
+          <t>Navegação issue</t>
+        </is>
+      </c>
+      <c r="U15" s="36" t="inlineStr">
+        <is>
+          <t>adb uiautomator dump indisponível neste ambiente; taps via coordenadas genéricas podem não ter alcançado elementos corretos. Validação real de navegação impossível.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="78" customHeight="1" s="58">
       <c r="A16" s="52" t="n">
@@ -22806,12 +23622,20 @@
       </c>
       <c r="R16" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S16" s="36" t="str"/>
-      <c r="T16" s="36" t="str"/>
-      <c r="U16" s="36" t="str"/>
+      <c r="T16" s="36" t="inlineStr">
+        <is>
+          <t>Acessibilidade issue</t>
+        </is>
+      </c>
+      <c r="U16" s="36" t="inlineStr">
+        <is>
+          <t>adb uiautomator dump indisponível neste ambiente; taps via coordenadas genéricas podem não ter alcançado elementos corretos. Validação real de navegação impossível.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="78" customHeight="1" s="58">
       <c r="A17" s="52" t="n">
@@ -22883,12 +23707,20 @@
       </c>
       <c r="R17" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="S17" s="36" t="str"/>
-      <c r="T17" s="36" t="str"/>
-      <c r="U17" s="36" t="str"/>
+      <c r="T17" s="36" t="inlineStr">
+        <is>
+          <t>Performance issue</t>
+        </is>
+      </c>
+      <c r="U17" s="36" t="inlineStr">
+        <is>
+          <t>adb uiautomator dump indisponível neste ambiente; taps via coordenadas genéricas podem não ter alcançado elementos corretos. Validação real de navegação impossível.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="78" customHeight="1" s="58">
       <c r="A18" s="52" t="n">
@@ -22962,11 +23794,15 @@
       </c>
       <c r="R18" s="52" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="S18" s="36" t="str"/>
-      <c r="T18" s="36" t="str"/>
+      <c r="T18" s="36" t="inlineStr">
+        <is>
+          <t>Relatório de E2E completo</t>
+        </is>
+      </c>
       <c r="U18" s="36" t="str"/>
     </row>
   </sheetData>

</xml_diff>